<commit_message>
Aanpassingen data processing zodat duidelijk
</commit_message>
<xml_diff>
--- a/Digital_Twin_Diabetes1/data/processed/run_003_input.xlsx
+++ b/Digital_Twin_Diabetes1/data/processed/run_003_input.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F182"/>
+  <dimension ref="A1:G182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,25 +424,30 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Glc</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>u</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ub</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>meal</t>
         </is>
@@ -452,19 +457,20 @@
       <c r="A2" t="n">
         <v>0</v>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
         <v>1990.243902439024</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>1</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -472,19 +478,20 @@
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
         <v>1.877</v>
       </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -492,9 +499,7 @@
       <c r="A4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>0</v>
       </c>
@@ -505,6 +510,9 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -512,9 +520,7 @@
       <c r="A5" t="n">
         <v>3</v>
       </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
         <v>0</v>
       </c>
@@ -525,6 +531,9 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -533,7 +542,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>12.1</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -545,6 +554,9 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -552,9 +564,7 @@
       <c r="A7" t="n">
         <v>5</v>
       </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
         <v>0</v>
       </c>
@@ -565,6 +575,9 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -572,19 +585,20 @@
       <c r="A8" t="n">
         <v>6</v>
       </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
         <v>1.715</v>
       </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -592,9 +606,7 @@
       <c r="A9" t="n">
         <v>7</v>
       </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
         <v>0</v>
       </c>
@@ -605,6 +617,9 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -612,9 +627,7 @@
       <c r="A10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
         <v>0</v>
       </c>
@@ -625,6 +638,9 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -633,7 +649,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>12.5</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
@@ -645,6 +661,9 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -652,9 +671,7 @@
       <c r="A12" t="n">
         <v>10</v>
       </c>
-      <c r="B12" t="n">
-        <v>0</v>
-      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
         <v>0</v>
       </c>
@@ -665,6 +682,9 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -672,19 +692,20 @@
       <c r="A13" t="n">
         <v>11</v>
       </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
         <v>1.149</v>
       </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -692,9 +713,7 @@
       <c r="A14" t="n">
         <v>12</v>
       </c>
-      <c r="B14" t="n">
-        <v>0</v>
-      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>0</v>
       </c>
@@ -705,6 +724,9 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -712,9 +734,7 @@
       <c r="A15" t="n">
         <v>13</v>
       </c>
-      <c r="B15" t="n">
-        <v>0</v>
-      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
         <v>0</v>
       </c>
@@ -725,6 +745,9 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -733,7 +756,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>12.4</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
@@ -745,6 +768,9 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -752,19 +778,20 @@
       <c r="A17" t="n">
         <v>15</v>
       </c>
-      <c r="B17" t="n">
-        <v>0</v>
-      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
         <v>2987.755102040816</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>1</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -772,19 +799,20 @@
       <c r="A18" t="n">
         <v>16</v>
       </c>
-      <c r="B18" t="n">
-        <v>0</v>
-      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
         <v>1.324</v>
       </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -792,9 +820,7 @@
       <c r="A19" t="n">
         <v>17</v>
       </c>
-      <c r="B19" t="n">
-        <v>0</v>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
         <v>0</v>
       </c>
@@ -805,6 +831,9 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -812,9 +841,7 @@
       <c r="A20" t="n">
         <v>18</v>
       </c>
-      <c r="B20" t="n">
-        <v>0</v>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
         <v>0</v>
       </c>
@@ -825,6 +852,9 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -833,7 +863,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>12.1</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
@@ -845,6 +875,9 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -852,9 +885,7 @@
       <c r="A22" t="n">
         <v>20</v>
       </c>
-      <c r="B22" t="n">
-        <v>0</v>
-      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
         <v>0</v>
       </c>
@@ -865,6 +896,9 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -872,19 +906,20 @@
       <c r="A23" t="n">
         <v>21</v>
       </c>
-      <c r="B23" t="n">
-        <v>0</v>
-      </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
         <v>1.053</v>
       </c>
-      <c r="D23" t="n">
-        <v>0</v>
-      </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -892,9 +927,7 @@
       <c r="A24" t="n">
         <v>22</v>
       </c>
-      <c r="B24" t="n">
-        <v>0</v>
-      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
         <v>0</v>
       </c>
@@ -905,6 +938,9 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -912,9 +948,7 @@
       <c r="A25" t="n">
         <v>23</v>
       </c>
-      <c r="B25" t="n">
-        <v>0</v>
-      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
         <v>0</v>
       </c>
@@ -925,6 +959,9 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -933,7 +970,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>12.1</v>
       </c>
       <c r="C26" t="n">
         <v>0</v>
@@ -945,6 +982,9 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -952,9 +992,7 @@
       <c r="A27" t="n">
         <v>25</v>
       </c>
-      <c r="B27" t="n">
-        <v>0</v>
-      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>0</v>
       </c>
@@ -965,6 +1003,9 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -972,19 +1013,20 @@
       <c r="A28" t="n">
         <v>26</v>
       </c>
-      <c r="B28" t="n">
-        <v>0</v>
-      </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
         <v>1.102</v>
       </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -992,9 +1034,7 @@
       <c r="A29" t="n">
         <v>27</v>
       </c>
-      <c r="B29" t="n">
-        <v>0</v>
-      </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
         <v>0</v>
       </c>
@@ -1005,6 +1045,9 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1012,9 +1055,7 @@
       <c r="A30" t="n">
         <v>28</v>
       </c>
-      <c r="B30" t="n">
-        <v>0</v>
-      </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
         <v>0</v>
       </c>
@@ -1025,6 +1066,9 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1033,7 +1077,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>11.9</v>
       </c>
       <c r="C31" t="n">
         <v>0</v>
@@ -1045,6 +1089,9 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1052,19 +1099,20 @@
       <c r="A32" t="n">
         <v>30</v>
       </c>
-      <c r="B32" t="n">
-        <v>0</v>
-      </c>
+      <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
         <v>6820</v>
       </c>
-      <c r="E32" t="n">
+      <c r="F32" t="n">
         <v>1</v>
       </c>
-      <c r="F32" t="n">
+      <c r="G32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1072,19 +1120,20 @@
       <c r="A33" t="n">
         <v>31</v>
       </c>
-      <c r="B33" t="n">
-        <v>0</v>
-      </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
         <v>0.65</v>
       </c>
-      <c r="D33" t="n">
-        <v>0</v>
-      </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1092,9 +1141,7 @@
       <c r="A34" t="n">
         <v>32</v>
       </c>
-      <c r="B34" t="n">
-        <v>0</v>
-      </c>
+      <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
         <v>0</v>
       </c>
@@ -1105,6 +1152,9 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1112,9 +1162,7 @@
       <c r="A35" t="n">
         <v>33</v>
       </c>
-      <c r="B35" t="n">
-        <v>0</v>
-      </c>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
         <v>0</v>
       </c>
@@ -1125,6 +1173,9 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1133,7 +1184,7 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>0</v>
+        <v>11.8</v>
       </c>
       <c r="C36" t="n">
         <v>0</v>
@@ -1145,6 +1196,9 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1152,9 +1206,7 @@
       <c r="A37" t="n">
         <v>35</v>
       </c>
-      <c r="B37" t="n">
-        <v>0</v>
-      </c>
+      <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
         <v>0</v>
       </c>
@@ -1165,6 +1217,9 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1172,9 +1227,7 @@
       <c r="A38" t="n">
         <v>36</v>
       </c>
-      <c r="B38" t="n">
-        <v>0</v>
-      </c>
+      <c r="B38" t="inlineStr"/>
       <c r="C38" t="n">
         <v>0</v>
       </c>
@@ -1185,6 +1238,9 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1192,9 +1248,7 @@
       <c r="A39" t="n">
         <v>37</v>
       </c>
-      <c r="B39" t="n">
-        <v>0</v>
-      </c>
+      <c r="B39" t="inlineStr"/>
       <c r="C39" t="n">
         <v>0</v>
       </c>
@@ -1205,6 +1259,9 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1212,9 +1269,7 @@
       <c r="A40" t="n">
         <v>38</v>
       </c>
-      <c r="B40" t="n">
-        <v>0</v>
-      </c>
+      <c r="B40" t="inlineStr"/>
       <c r="C40" t="n">
         <v>0</v>
       </c>
@@ -1225,6 +1280,9 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1233,7 +1291,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>0</v>
+        <v>11.6</v>
       </c>
       <c r="C41" t="n">
         <v>0</v>
@@ -1245,6 +1303,9 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1252,9 +1313,7 @@
       <c r="A42" t="n">
         <v>40</v>
       </c>
-      <c r="B42" t="n">
-        <v>0</v>
-      </c>
+      <c r="B42" t="inlineStr"/>
       <c r="C42" t="n">
         <v>0</v>
       </c>
@@ -1265,6 +1324,9 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1272,9 +1334,7 @@
       <c r="A43" t="n">
         <v>41</v>
       </c>
-      <c r="B43" t="n">
-        <v>0</v>
-      </c>
+      <c r="B43" t="inlineStr"/>
       <c r="C43" t="n">
         <v>0</v>
       </c>
@@ -1285,6 +1345,9 @@
         <v>0</v>
       </c>
       <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1292,9 +1355,7 @@
       <c r="A44" t="n">
         <v>42</v>
       </c>
-      <c r="B44" t="n">
-        <v>0</v>
-      </c>
+      <c r="B44" t="inlineStr"/>
       <c r="C44" t="n">
         <v>0</v>
       </c>
@@ -1305,6 +1366,9 @@
         <v>0</v>
       </c>
       <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1312,9 +1376,7 @@
       <c r="A45" t="n">
         <v>43</v>
       </c>
-      <c r="B45" t="n">
-        <v>0</v>
-      </c>
+      <c r="B45" t="inlineStr"/>
       <c r="C45" t="n">
         <v>0</v>
       </c>
@@ -1325,6 +1387,9 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1333,7 +1398,7 @@
         <v>44</v>
       </c>
       <c r="B46" t="n">
-        <v>0</v>
+        <v>11.4</v>
       </c>
       <c r="C46" t="n">
         <v>0</v>
@@ -1345,6 +1410,9 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1352,19 +1420,20 @@
       <c r="A47" t="n">
         <v>45</v>
       </c>
-      <c r="B47" t="n">
-        <v>0</v>
-      </c>
+      <c r="B47" t="inlineStr"/>
       <c r="C47" t="n">
         <v>0</v>
       </c>
       <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
         <v>6456.25</v>
       </c>
-      <c r="E47" t="n">
+      <c r="F47" t="n">
         <v>1</v>
       </c>
-      <c r="F47" t="n">
+      <c r="G47" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1372,9 +1441,7 @@
       <c r="A48" t="n">
         <v>46</v>
       </c>
-      <c r="B48" t="n">
-        <v>0</v>
-      </c>
+      <c r="B48" t="inlineStr"/>
       <c r="C48" t="n">
         <v>0</v>
       </c>
@@ -1385,6 +1452,9 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1392,9 +1462,7 @@
       <c r="A49" t="n">
         <v>47</v>
       </c>
-      <c r="B49" t="n">
-        <v>0</v>
-      </c>
+      <c r="B49" t="inlineStr"/>
       <c r="C49" t="n">
         <v>0</v>
       </c>
@@ -1405,6 +1473,9 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1412,9 +1483,7 @@
       <c r="A50" t="n">
         <v>48</v>
       </c>
-      <c r="B50" t="n">
-        <v>0</v>
-      </c>
+      <c r="B50" t="inlineStr"/>
       <c r="C50" t="n">
         <v>0</v>
       </c>
@@ -1425,6 +1494,9 @@
         <v>0</v>
       </c>
       <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1433,7 +1505,7 @@
         <v>49</v>
       </c>
       <c r="B51" t="n">
-        <v>0</v>
+        <v>11.3</v>
       </c>
       <c r="C51" t="n">
         <v>0</v>
@@ -1445,6 +1517,9 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1452,9 +1527,7 @@
       <c r="A52" t="n">
         <v>50</v>
       </c>
-      <c r="B52" t="n">
-        <v>0</v>
-      </c>
+      <c r="B52" t="inlineStr"/>
       <c r="C52" t="n">
         <v>0</v>
       </c>
@@ -1465,6 +1538,9 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1472,12 +1548,10 @@
       <c r="A53" t="n">
         <v>51</v>
       </c>
-      <c r="B53" t="n">
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="n">
         <v>0.083</v>
       </c>
-      <c r="C53" t="n">
-        <v>0</v>
-      </c>
       <c r="D53" t="n">
         <v>0</v>
       </c>
@@ -1485,6 +1559,9 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1492,9 +1569,7 @@
       <c r="A54" t="n">
         <v>52</v>
       </c>
-      <c r="B54" t="n">
-        <v>0</v>
-      </c>
+      <c r="B54" t="inlineStr"/>
       <c r="C54" t="n">
         <v>0</v>
       </c>
@@ -1505,6 +1580,9 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1512,9 +1590,7 @@
       <c r="A55" t="n">
         <v>53</v>
       </c>
-      <c r="B55" t="n">
-        <v>0</v>
-      </c>
+      <c r="B55" t="inlineStr"/>
       <c r="C55" t="n">
         <v>0</v>
       </c>
@@ -1525,6 +1601,9 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1533,7 +1612,7 @@
         <v>54</v>
       </c>
       <c r="B56" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
       <c r="C56" t="n">
         <v>0</v>
@@ -1545,6 +1624,9 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1552,9 +1634,7 @@
       <c r="A57" t="n">
         <v>55</v>
       </c>
-      <c r="B57" t="n">
-        <v>0</v>
-      </c>
+      <c r="B57" t="inlineStr"/>
       <c r="C57" t="n">
         <v>0</v>
       </c>
@@ -1565,6 +1645,9 @@
         <v>0</v>
       </c>
       <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1572,9 +1655,7 @@
       <c r="A58" t="n">
         <v>56</v>
       </c>
-      <c r="B58" t="n">
-        <v>0</v>
-      </c>
+      <c r="B58" t="inlineStr"/>
       <c r="C58" t="n">
         <v>0</v>
       </c>
@@ -1585,6 +1666,9 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1592,9 +1676,7 @@
       <c r="A59" t="n">
         <v>57</v>
       </c>
-      <c r="B59" t="n">
-        <v>0</v>
-      </c>
+      <c r="B59" t="inlineStr"/>
       <c r="C59" t="n">
         <v>0</v>
       </c>
@@ -1605,6 +1687,9 @@
         <v>0</v>
       </c>
       <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1612,9 +1697,7 @@
       <c r="A60" t="n">
         <v>58</v>
       </c>
-      <c r="B60" t="n">
-        <v>0</v>
-      </c>
+      <c r="B60" t="inlineStr"/>
       <c r="C60" t="n">
         <v>0</v>
       </c>
@@ -1625,6 +1708,9 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1633,7 +1719,7 @@
         <v>59</v>
       </c>
       <c r="B61" t="n">
-        <v>0</v>
+        <v>10.2</v>
       </c>
       <c r="C61" t="n">
         <v>0</v>
@@ -1645,6 +1731,9 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1652,19 +1741,20 @@
       <c r="A62" t="n">
         <v>60</v>
       </c>
-      <c r="B62" t="n">
-        <v>0</v>
-      </c>
+      <c r="B62" t="inlineStr"/>
       <c r="C62" t="n">
         <v>0</v>
       </c>
       <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="n">
         <v>4015.384615384615</v>
       </c>
-      <c r="E62" t="n">
+      <c r="F62" t="n">
         <v>1</v>
       </c>
-      <c r="F62" t="n">
+      <c r="G62" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1672,9 +1762,7 @@
       <c r="A63" t="n">
         <v>61</v>
       </c>
-      <c r="B63" t="n">
-        <v>0</v>
-      </c>
+      <c r="B63" t="inlineStr"/>
       <c r="C63" t="n">
         <v>0</v>
       </c>
@@ -1685,6 +1773,9 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1692,9 +1783,7 @@
       <c r="A64" t="n">
         <v>62</v>
       </c>
-      <c r="B64" t="n">
-        <v>0</v>
-      </c>
+      <c r="B64" t="inlineStr"/>
       <c r="C64" t="n">
         <v>0</v>
       </c>
@@ -1705,6 +1794,9 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1712,9 +1804,7 @@
       <c r="A65" t="n">
         <v>63</v>
       </c>
-      <c r="B65" t="n">
-        <v>0</v>
-      </c>
+      <c r="B65" t="inlineStr"/>
       <c r="C65" t="n">
         <v>0</v>
       </c>
@@ -1725,6 +1815,9 @@
         <v>0</v>
       </c>
       <c r="F65" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1733,7 +1826,7 @@
         <v>64</v>
       </c>
       <c r="B66" t="n">
-        <v>0</v>
+        <v>9.4</v>
       </c>
       <c r="C66" t="n">
         <v>0</v>
@@ -1745,6 +1838,9 @@
         <v>0</v>
       </c>
       <c r="F66" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1752,9 +1848,7 @@
       <c r="A67" t="n">
         <v>65</v>
       </c>
-      <c r="B67" t="n">
-        <v>0</v>
-      </c>
+      <c r="B67" t="inlineStr"/>
       <c r="C67" t="n">
         <v>0</v>
       </c>
@@ -1765,6 +1859,9 @@
         <v>0</v>
       </c>
       <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1772,9 +1869,7 @@
       <c r="A68" t="n">
         <v>66</v>
       </c>
-      <c r="B68" t="n">
-        <v>0</v>
-      </c>
+      <c r="B68" t="inlineStr"/>
       <c r="C68" t="n">
         <v>0</v>
       </c>
@@ -1785,6 +1880,9 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1792,9 +1890,7 @@
       <c r="A69" t="n">
         <v>67</v>
       </c>
-      <c r="B69" t="n">
-        <v>0</v>
-      </c>
+      <c r="B69" t="inlineStr"/>
       <c r="C69" t="n">
         <v>0</v>
       </c>
@@ -1805,6 +1901,9 @@
         <v>0</v>
       </c>
       <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1812,9 +1911,7 @@
       <c r="A70" t="n">
         <v>68</v>
       </c>
-      <c r="B70" t="n">
-        <v>0</v>
-      </c>
+      <c r="B70" t="inlineStr"/>
       <c r="C70" t="n">
         <v>0</v>
       </c>
@@ -1825,6 +1922,9 @@
         <v>0</v>
       </c>
       <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1833,7 +1933,7 @@
         <v>69</v>
       </c>
       <c r="B71" t="n">
-        <v>0</v>
+        <v>8.9</v>
       </c>
       <c r="C71" t="n">
         <v>0</v>
@@ -1845,6 +1945,9 @@
         <v>0</v>
       </c>
       <c r="F71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1852,9 +1955,7 @@
       <c r="A72" t="n">
         <v>70</v>
       </c>
-      <c r="B72" t="n">
-        <v>0</v>
-      </c>
+      <c r="B72" t="inlineStr"/>
       <c r="C72" t="n">
         <v>0</v>
       </c>
@@ -1865,6 +1966,9 @@
         <v>0</v>
       </c>
       <c r="F72" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1872,19 +1976,20 @@
       <c r="A73" t="n">
         <v>71</v>
       </c>
-      <c r="B73" t="n">
-        <v>0</v>
-      </c>
+      <c r="B73" t="inlineStr"/>
       <c r="C73" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" t="n">
         <v>0.236</v>
       </c>
-      <c r="D73" t="n">
-        <v>0</v>
-      </c>
       <c r="E73" t="n">
         <v>0</v>
       </c>
       <c r="F73" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1892,9 +1997,7 @@
       <c r="A74" t="n">
         <v>72</v>
       </c>
-      <c r="B74" t="n">
-        <v>0</v>
-      </c>
+      <c r="B74" t="inlineStr"/>
       <c r="C74" t="n">
         <v>0</v>
       </c>
@@ -1905,6 +2008,9 @@
         <v>0</v>
       </c>
       <c r="F74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1912,9 +2018,7 @@
       <c r="A75" t="n">
         <v>73</v>
       </c>
-      <c r="B75" t="n">
-        <v>0</v>
-      </c>
+      <c r="B75" t="inlineStr"/>
       <c r="C75" t="n">
         <v>0</v>
       </c>
@@ -1925,6 +2029,9 @@
         <v>0</v>
       </c>
       <c r="F75" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1933,7 +2040,7 @@
         <v>74</v>
       </c>
       <c r="B76" t="n">
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="C76" t="n">
         <v>0</v>
@@ -1945,6 +2052,9 @@
         <v>0</v>
       </c>
       <c r="F76" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1952,19 +2062,20 @@
       <c r="A77" t="n">
         <v>75</v>
       </c>
-      <c r="B77" t="n">
-        <v>0</v>
-      </c>
+      <c r="B77" t="inlineStr"/>
       <c r="C77" t="n">
         <v>0</v>
       </c>
       <c r="D77" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" t="n">
         <v>3658.333333333333</v>
       </c>
-      <c r="E77" t="n">
+      <c r="F77" t="n">
         <v>1</v>
       </c>
-      <c r="F77" t="n">
+      <c r="G77" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1972,19 +2083,20 @@
       <c r="A78" t="n">
         <v>76</v>
       </c>
-      <c r="B78" t="n">
-        <v>0</v>
-      </c>
+      <c r="B78" t="inlineStr"/>
       <c r="C78" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" t="n">
         <v>0.108</v>
       </c>
-      <c r="D78" t="n">
-        <v>0</v>
-      </c>
       <c r="E78" t="n">
         <v>0</v>
       </c>
       <c r="F78" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1992,9 +2104,7 @@
       <c r="A79" t="n">
         <v>77</v>
       </c>
-      <c r="B79" t="n">
-        <v>0</v>
-      </c>
+      <c r="B79" t="inlineStr"/>
       <c r="C79" t="n">
         <v>0</v>
       </c>
@@ -2005,6 +2115,9 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2012,9 +2125,7 @@
       <c r="A80" t="n">
         <v>78</v>
       </c>
-      <c r="B80" t="n">
-        <v>0</v>
-      </c>
+      <c r="B80" t="inlineStr"/>
       <c r="C80" t="n">
         <v>0</v>
       </c>
@@ -2025,6 +2136,9 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2033,7 +2147,7 @@
         <v>79</v>
       </c>
       <c r="B81" t="n">
-        <v>0</v>
+        <v>8.1</v>
       </c>
       <c r="C81" t="n">
         <v>0</v>
@@ -2045,6 +2159,9 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2052,9 +2169,7 @@
       <c r="A82" t="n">
         <v>80</v>
       </c>
-      <c r="B82" t="n">
-        <v>0</v>
-      </c>
+      <c r="B82" t="inlineStr"/>
       <c r="C82" t="n">
         <v>0</v>
       </c>
@@ -2065,6 +2180,9 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2072,19 +2190,20 @@
       <c r="A83" t="n">
         <v>81</v>
       </c>
-      <c r="B83" t="n">
-        <v>0</v>
-      </c>
+      <c r="B83" t="inlineStr"/>
       <c r="C83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" t="n">
         <v>0.1</v>
       </c>
-      <c r="D83" t="n">
-        <v>0</v>
-      </c>
       <c r="E83" t="n">
         <v>0</v>
       </c>
       <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2092,9 +2211,7 @@
       <c r="A84" t="n">
         <v>82</v>
       </c>
-      <c r="B84" t="n">
-        <v>0</v>
-      </c>
+      <c r="B84" t="inlineStr"/>
       <c r="C84" t="n">
         <v>0</v>
       </c>
@@ -2105,6 +2222,9 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2112,9 +2232,7 @@
       <c r="A85" t="n">
         <v>83</v>
       </c>
-      <c r="B85" t="n">
-        <v>0</v>
-      </c>
+      <c r="B85" t="inlineStr"/>
       <c r="C85" t="n">
         <v>0</v>
       </c>
@@ -2125,6 +2243,9 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2133,7 +2254,7 @@
         <v>84</v>
       </c>
       <c r="B86" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="C86" t="n">
         <v>0</v>
@@ -2145,6 +2266,9 @@
         <v>0</v>
       </c>
       <c r="F86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2152,9 +2276,7 @@
       <c r="A87" t="n">
         <v>85</v>
       </c>
-      <c r="B87" t="n">
-        <v>0</v>
-      </c>
+      <c r="B87" t="inlineStr"/>
       <c r="C87" t="n">
         <v>0</v>
       </c>
@@ -2165,6 +2287,9 @@
         <v>0</v>
       </c>
       <c r="F87" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2172,9 +2297,7 @@
       <c r="A88" t="n">
         <v>86</v>
       </c>
-      <c r="B88" t="n">
-        <v>0</v>
-      </c>
+      <c r="B88" t="inlineStr"/>
       <c r="C88" t="n">
         <v>0</v>
       </c>
@@ -2185,6 +2308,9 @@
         <v>0</v>
       </c>
       <c r="F88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2192,9 +2318,7 @@
       <c r="A89" t="n">
         <v>87</v>
       </c>
-      <c r="B89" t="n">
-        <v>0</v>
-      </c>
+      <c r="B89" t="inlineStr"/>
       <c r="C89" t="n">
         <v>0</v>
       </c>
@@ -2205,6 +2329,9 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2212,9 +2339,7 @@
       <c r="A90" t="n">
         <v>88</v>
       </c>
-      <c r="B90" t="n">
-        <v>0</v>
-      </c>
+      <c r="B90" t="inlineStr"/>
       <c r="C90" t="n">
         <v>0</v>
       </c>
@@ -2225,6 +2350,9 @@
         <v>0</v>
       </c>
       <c r="F90" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2233,7 +2361,7 @@
         <v>89</v>
       </c>
       <c r="B91" t="n">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="C91" t="n">
         <v>0</v>
@@ -2245,6 +2373,9 @@
         <v>0</v>
       </c>
       <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2252,19 +2383,20 @@
       <c r="A92" t="n">
         <v>90</v>
       </c>
-      <c r="B92" t="n">
-        <v>0</v>
-      </c>
+      <c r="B92" t="inlineStr"/>
       <c r="C92" t="n">
         <v>0</v>
       </c>
       <c r="D92" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" t="n">
         <v>750</v>
       </c>
-      <c r="E92" t="n">
+      <c r="F92" t="n">
         <v>1</v>
       </c>
-      <c r="F92" t="n">
+      <c r="G92" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2272,9 +2404,7 @@
       <c r="A93" t="n">
         <v>91</v>
       </c>
-      <c r="B93" t="n">
-        <v>0</v>
-      </c>
+      <c r="B93" t="inlineStr"/>
       <c r="C93" t="n">
         <v>0</v>
       </c>
@@ -2285,6 +2415,9 @@
         <v>0</v>
       </c>
       <c r="F93" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2292,9 +2425,7 @@
       <c r="A94" t="n">
         <v>92</v>
       </c>
-      <c r="B94" t="n">
-        <v>0</v>
-      </c>
+      <c r="B94" t="inlineStr"/>
       <c r="C94" t="n">
         <v>0</v>
       </c>
@@ -2305,6 +2436,9 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2312,9 +2446,7 @@
       <c r="A95" t="n">
         <v>93</v>
       </c>
-      <c r="B95" t="n">
-        <v>0</v>
-      </c>
+      <c r="B95" t="inlineStr"/>
       <c r="C95" t="n">
         <v>0</v>
       </c>
@@ -2325,6 +2457,9 @@
         <v>0</v>
       </c>
       <c r="F95" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2333,7 +2468,7 @@
         <v>94</v>
       </c>
       <c r="B96" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="C96" t="n">
         <v>0</v>
@@ -2345,6 +2480,9 @@
         <v>0</v>
       </c>
       <c r="F96" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2352,9 +2490,7 @@
       <c r="A97" t="n">
         <v>95</v>
       </c>
-      <c r="B97" t="n">
-        <v>0</v>
-      </c>
+      <c r="B97" t="inlineStr"/>
       <c r="C97" t="n">
         <v>0</v>
       </c>
@@ -2365,6 +2501,9 @@
         <v>0</v>
       </c>
       <c r="F97" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2372,9 +2511,7 @@
       <c r="A98" t="n">
         <v>96</v>
       </c>
-      <c r="B98" t="n">
-        <v>0</v>
-      </c>
+      <c r="B98" t="inlineStr"/>
       <c r="C98" t="n">
         <v>0</v>
       </c>
@@ -2385,6 +2522,9 @@
         <v>0</v>
       </c>
       <c r="F98" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2392,9 +2532,7 @@
       <c r="A99" t="n">
         <v>97</v>
       </c>
-      <c r="B99" t="n">
-        <v>0</v>
-      </c>
+      <c r="B99" t="inlineStr"/>
       <c r="C99" t="n">
         <v>0</v>
       </c>
@@ -2405,6 +2543,9 @@
         <v>0</v>
       </c>
       <c r="F99" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2412,9 +2553,7 @@
       <c r="A100" t="n">
         <v>98</v>
       </c>
-      <c r="B100" t="n">
-        <v>0</v>
-      </c>
+      <c r="B100" t="inlineStr"/>
       <c r="C100" t="n">
         <v>0</v>
       </c>
@@ -2425,6 +2564,9 @@
         <v>0</v>
       </c>
       <c r="F100" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2433,7 +2575,7 @@
         <v>99</v>
       </c>
       <c r="B101" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="C101" t="n">
         <v>0</v>
@@ -2445,6 +2587,9 @@
         <v>0</v>
       </c>
       <c r="F101" t="n">
+        <v>0</v>
+      </c>
+      <c r="G101" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2452,9 +2597,7 @@
       <c r="A102" t="n">
         <v>100</v>
       </c>
-      <c r="B102" t="n">
-        <v>0</v>
-      </c>
+      <c r="B102" t="inlineStr"/>
       <c r="C102" t="n">
         <v>0</v>
       </c>
@@ -2465,6 +2608,9 @@
         <v>0</v>
       </c>
       <c r="F102" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2472,9 +2618,7 @@
       <c r="A103" t="n">
         <v>101</v>
       </c>
-      <c r="B103" t="n">
-        <v>0</v>
-      </c>
+      <c r="B103" t="inlineStr"/>
       <c r="C103" t="n">
         <v>0</v>
       </c>
@@ -2485,6 +2629,9 @@
         <v>0</v>
       </c>
       <c r="F103" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2492,9 +2639,7 @@
       <c r="A104" t="n">
         <v>102</v>
       </c>
-      <c r="B104" t="n">
-        <v>0</v>
-      </c>
+      <c r="B104" t="inlineStr"/>
       <c r="C104" t="n">
         <v>0</v>
       </c>
@@ -2505,6 +2650,9 @@
         <v>0</v>
       </c>
       <c r="F104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2512,9 +2660,7 @@
       <c r="A105" t="n">
         <v>103</v>
       </c>
-      <c r="B105" t="n">
-        <v>0</v>
-      </c>
+      <c r="B105" t="inlineStr"/>
       <c r="C105" t="n">
         <v>0</v>
       </c>
@@ -2525,6 +2671,9 @@
         <v>0</v>
       </c>
       <c r="F105" t="n">
+        <v>0</v>
+      </c>
+      <c r="G105" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2533,7 +2682,7 @@
         <v>104</v>
       </c>
       <c r="B106" t="n">
-        <v>0</v>
+        <v>6.6</v>
       </c>
       <c r="C106" t="n">
         <v>0</v>
@@ -2545,6 +2694,9 @@
         <v>0</v>
       </c>
       <c r="F106" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2552,19 +2704,20 @@
       <c r="A107" t="n">
         <v>105</v>
       </c>
-      <c r="B107" t="n">
-        <v>0</v>
-      </c>
+      <c r="B107" t="inlineStr"/>
       <c r="C107" t="n">
         <v>0</v>
       </c>
       <c r="D107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" t="n">
         <v>1150</v>
       </c>
-      <c r="E107" t="n">
+      <c r="F107" t="n">
         <v>1</v>
       </c>
-      <c r="F107" t="n">
+      <c r="G107" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2572,9 +2725,7 @@
       <c r="A108" t="n">
         <v>106</v>
       </c>
-      <c r="B108" t="n">
-        <v>0</v>
-      </c>
+      <c r="B108" t="inlineStr"/>
       <c r="C108" t="n">
         <v>0</v>
       </c>
@@ -2585,6 +2736,9 @@
         <v>0</v>
       </c>
       <c r="F108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2592,9 +2746,7 @@
       <c r="A109" t="n">
         <v>107</v>
       </c>
-      <c r="B109" t="n">
-        <v>0</v>
-      </c>
+      <c r="B109" t="inlineStr"/>
       <c r="C109" t="n">
         <v>0</v>
       </c>
@@ -2605,6 +2757,9 @@
         <v>0</v>
       </c>
       <c r="F109" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2612,9 +2767,7 @@
       <c r="A110" t="n">
         <v>108</v>
       </c>
-      <c r="B110" t="n">
-        <v>0</v>
-      </c>
+      <c r="B110" t="inlineStr"/>
       <c r="C110" t="n">
         <v>0</v>
       </c>
@@ -2625,6 +2778,9 @@
         <v>0</v>
       </c>
       <c r="F110" t="n">
+        <v>0</v>
+      </c>
+      <c r="G110" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2633,7 +2789,7 @@
         <v>109</v>
       </c>
       <c r="B111" t="n">
-        <v>0</v>
+        <v>6.3</v>
       </c>
       <c r="C111" t="n">
         <v>0</v>
@@ -2645,6 +2801,9 @@
         <v>0</v>
       </c>
       <c r="F111" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2652,9 +2811,7 @@
       <c r="A112" t="n">
         <v>110</v>
       </c>
-      <c r="B112" t="n">
-        <v>0</v>
-      </c>
+      <c r="B112" t="inlineStr"/>
       <c r="C112" t="n">
         <v>0</v>
       </c>
@@ -2665,6 +2822,9 @@
         <v>0</v>
       </c>
       <c r="F112" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2672,9 +2832,7 @@
       <c r="A113" t="n">
         <v>111</v>
       </c>
-      <c r="B113" t="n">
-        <v>0</v>
-      </c>
+      <c r="B113" t="inlineStr"/>
       <c r="C113" t="n">
         <v>0</v>
       </c>
@@ -2685,6 +2843,9 @@
         <v>0</v>
       </c>
       <c r="F113" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2692,12 +2853,10 @@
       <c r="A114" t="n">
         <v>112</v>
       </c>
-      <c r="B114" t="n">
+      <c r="B114" t="inlineStr"/>
+      <c r="C114" t="n">
         <v>6.36</v>
       </c>
-      <c r="C114" t="n">
-        <v>0</v>
-      </c>
       <c r="D114" t="n">
         <v>0</v>
       </c>
@@ -2705,6 +2864,9 @@
         <v>0</v>
       </c>
       <c r="F114" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" t="n">
         <v>47</v>
       </c>
     </row>
@@ -2712,9 +2874,7 @@
       <c r="A115" t="n">
         <v>113</v>
       </c>
-      <c r="B115" t="n">
-        <v>0</v>
-      </c>
+      <c r="B115" t="inlineStr"/>
       <c r="C115" t="n">
         <v>0</v>
       </c>
@@ -2725,6 +2885,9 @@
         <v>0</v>
       </c>
       <c r="F115" t="n">
+        <v>0</v>
+      </c>
+      <c r="G115" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2733,7 +2896,7 @@
         <v>114</v>
       </c>
       <c r="B116" t="n">
-        <v>0</v>
+        <v>6.2</v>
       </c>
       <c r="C116" t="n">
         <v>0</v>
@@ -2745,6 +2908,9 @@
         <v>0</v>
       </c>
       <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2752,9 +2918,7 @@
       <c r="A117" t="n">
         <v>115</v>
       </c>
-      <c r="B117" t="n">
-        <v>0</v>
-      </c>
+      <c r="B117" t="inlineStr"/>
       <c r="C117" t="n">
         <v>0</v>
       </c>
@@ -2765,6 +2929,9 @@
         <v>0</v>
       </c>
       <c r="F117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2772,19 +2939,20 @@
       <c r="A118" t="n">
         <v>116</v>
       </c>
-      <c r="B118" t="n">
-        <v>0</v>
-      </c>
+      <c r="B118" t="inlineStr"/>
       <c r="C118" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" t="n">
         <v>0.3</v>
       </c>
-      <c r="D118" t="n">
-        <v>0</v>
-      </c>
       <c r="E118" t="n">
         <v>0</v>
       </c>
       <c r="F118" t="n">
+        <v>0</v>
+      </c>
+      <c r="G118" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2792,9 +2960,7 @@
       <c r="A119" t="n">
         <v>117</v>
       </c>
-      <c r="B119" t="n">
-        <v>0</v>
-      </c>
+      <c r="B119" t="inlineStr"/>
       <c r="C119" t="n">
         <v>0</v>
       </c>
@@ -2805,6 +2971,9 @@
         <v>0</v>
       </c>
       <c r="F119" t="n">
+        <v>0</v>
+      </c>
+      <c r="G119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2812,9 +2981,7 @@
       <c r="A120" t="n">
         <v>118</v>
       </c>
-      <c r="B120" t="n">
-        <v>0</v>
-      </c>
+      <c r="B120" t="inlineStr"/>
       <c r="C120" t="n">
         <v>0</v>
       </c>
@@ -2825,6 +2992,9 @@
         <v>0</v>
       </c>
       <c r="F120" t="n">
+        <v>0</v>
+      </c>
+      <c r="G120" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2833,7 +3003,7 @@
         <v>119</v>
       </c>
       <c r="B121" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="C121" t="n">
         <v>0</v>
@@ -2845,6 +3015,9 @@
         <v>0</v>
       </c>
       <c r="F121" t="n">
+        <v>0</v>
+      </c>
+      <c r="G121" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2852,9 +3025,7 @@
       <c r="A122" t="n">
         <v>120</v>
       </c>
-      <c r="B122" t="n">
-        <v>0</v>
-      </c>
+      <c r="B122" t="inlineStr"/>
       <c r="C122" t="n">
         <v>0</v>
       </c>
@@ -2865,6 +3036,9 @@
         <v>0</v>
       </c>
       <c r="F122" t="n">
+        <v>0</v>
+      </c>
+      <c r="G122" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2872,19 +3046,20 @@
       <c r="A123" t="n">
         <v>121</v>
       </c>
-      <c r="B123" t="n">
-        <v>0</v>
-      </c>
+      <c r="B123" t="inlineStr"/>
       <c r="C123" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" t="n">
         <v>0.486</v>
       </c>
-      <c r="D123" t="n">
-        <v>0</v>
-      </c>
       <c r="E123" t="n">
         <v>0</v>
       </c>
       <c r="F123" t="n">
+        <v>0</v>
+      </c>
+      <c r="G123" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2892,9 +3067,7 @@
       <c r="A124" t="n">
         <v>122</v>
       </c>
-      <c r="B124" t="n">
-        <v>0</v>
-      </c>
+      <c r="B124" t="inlineStr"/>
       <c r="C124" t="n">
         <v>0</v>
       </c>
@@ -2905,6 +3078,9 @@
         <v>0</v>
       </c>
       <c r="F124" t="n">
+        <v>0</v>
+      </c>
+      <c r="G124" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2912,9 +3088,7 @@
       <c r="A125" t="n">
         <v>123</v>
       </c>
-      <c r="B125" t="n">
-        <v>0</v>
-      </c>
+      <c r="B125" t="inlineStr"/>
       <c r="C125" t="n">
         <v>0</v>
       </c>
@@ -2925,6 +3099,9 @@
         <v>0</v>
       </c>
       <c r="F125" t="n">
+        <v>0</v>
+      </c>
+      <c r="G125" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2933,7 +3110,7 @@
         <v>124</v>
       </c>
       <c r="B126" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="C126" t="n">
         <v>0</v>
@@ -2945,6 +3122,9 @@
         <v>0</v>
       </c>
       <c r="F126" t="n">
+        <v>0</v>
+      </c>
+      <c r="G126" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2952,9 +3132,7 @@
       <c r="A127" t="n">
         <v>125</v>
       </c>
-      <c r="B127" t="n">
-        <v>0</v>
-      </c>
+      <c r="B127" t="inlineStr"/>
       <c r="C127" t="n">
         <v>0</v>
       </c>
@@ -2965,6 +3143,9 @@
         <v>0</v>
       </c>
       <c r="F127" t="n">
+        <v>0</v>
+      </c>
+      <c r="G127" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2972,19 +3153,20 @@
       <c r="A128" t="n">
         <v>126</v>
       </c>
-      <c r="B128" t="n">
-        <v>0</v>
-      </c>
+      <c r="B128" t="inlineStr"/>
       <c r="C128" t="n">
+        <v>0</v>
+      </c>
+      <c r="D128" t="n">
         <v>0.607</v>
       </c>
-      <c r="D128" t="n">
-        <v>0</v>
-      </c>
       <c r="E128" t="n">
         <v>0</v>
       </c>
       <c r="F128" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2992,9 +3174,7 @@
       <c r="A129" t="n">
         <v>127</v>
       </c>
-      <c r="B129" t="n">
-        <v>0</v>
-      </c>
+      <c r="B129" t="inlineStr"/>
       <c r="C129" t="n">
         <v>0</v>
       </c>
@@ -3005,6 +3185,9 @@
         <v>0</v>
       </c>
       <c r="F129" t="n">
+        <v>0</v>
+      </c>
+      <c r="G129" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3012,9 +3195,7 @@
       <c r="A130" t="n">
         <v>128</v>
       </c>
-      <c r="B130" t="n">
-        <v>0</v>
-      </c>
+      <c r="B130" t="inlineStr"/>
       <c r="C130" t="n">
         <v>0</v>
       </c>
@@ -3025,6 +3206,9 @@
         <v>0</v>
       </c>
       <c r="F130" t="n">
+        <v>0</v>
+      </c>
+      <c r="G130" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3033,7 +3217,7 @@
         <v>129</v>
       </c>
       <c r="B131" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="C131" t="n">
         <v>0</v>
@@ -3045,6 +3229,9 @@
         <v>0</v>
       </c>
       <c r="F131" t="n">
+        <v>0</v>
+      </c>
+      <c r="G131" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3052,9 +3239,7 @@
       <c r="A132" t="n">
         <v>130</v>
       </c>
-      <c r="B132" t="n">
-        <v>0</v>
-      </c>
+      <c r="B132" t="inlineStr"/>
       <c r="C132" t="n">
         <v>0</v>
       </c>
@@ -3065,6 +3250,9 @@
         <v>0</v>
       </c>
       <c r="F132" t="n">
+        <v>0</v>
+      </c>
+      <c r="G132" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3072,19 +3260,20 @@
       <c r="A133" t="n">
         <v>131</v>
       </c>
-      <c r="B133" t="n">
-        <v>0</v>
-      </c>
+      <c r="B133" t="inlineStr"/>
       <c r="C133" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" t="n">
         <v>0.7</v>
       </c>
-      <c r="D133" t="n">
-        <v>0</v>
-      </c>
       <c r="E133" t="n">
         <v>0</v>
       </c>
       <c r="F133" t="n">
+        <v>0</v>
+      </c>
+      <c r="G133" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3092,9 +3281,7 @@
       <c r="A134" t="n">
         <v>132</v>
       </c>
-      <c r="B134" t="n">
-        <v>0</v>
-      </c>
+      <c r="B134" t="inlineStr"/>
       <c r="C134" t="n">
         <v>0</v>
       </c>
@@ -3105,6 +3292,9 @@
         <v>0</v>
       </c>
       <c r="F134" t="n">
+        <v>0</v>
+      </c>
+      <c r="G134" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3112,9 +3302,7 @@
       <c r="A135" t="n">
         <v>133</v>
       </c>
-      <c r="B135" t="n">
-        <v>0</v>
-      </c>
+      <c r="B135" t="inlineStr"/>
       <c r="C135" t="n">
         <v>0</v>
       </c>
@@ -3125,6 +3313,9 @@
         <v>0</v>
       </c>
       <c r="F135" t="n">
+        <v>0</v>
+      </c>
+      <c r="G135" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3133,7 +3324,7 @@
         <v>134</v>
       </c>
       <c r="B136" t="n">
-        <v>0</v>
+        <v>5.8</v>
       </c>
       <c r="C136" t="n">
         <v>0</v>
@@ -3145,6 +3336,9 @@
         <v>0</v>
       </c>
       <c r="F136" t="n">
+        <v>0</v>
+      </c>
+      <c r="G136" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3152,19 +3346,20 @@
       <c r="A137" t="n">
         <v>135</v>
       </c>
-      <c r="B137" t="n">
-        <v>0</v>
-      </c>
+      <c r="B137" t="inlineStr"/>
       <c r="C137" t="n">
         <v>0</v>
       </c>
       <c r="D137" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" t="n">
         <v>525</v>
       </c>
-      <c r="E137" t="n">
+      <c r="F137" t="n">
         <v>1</v>
       </c>
-      <c r="F137" t="n">
+      <c r="G137" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3172,9 +3367,7 @@
       <c r="A138" t="n">
         <v>136</v>
       </c>
-      <c r="B138" t="n">
-        <v>0</v>
-      </c>
+      <c r="B138" t="inlineStr"/>
       <c r="C138" t="n">
         <v>0</v>
       </c>
@@ -3185,6 +3378,9 @@
         <v>0</v>
       </c>
       <c r="F138" t="n">
+        <v>0</v>
+      </c>
+      <c r="G138" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3192,9 +3388,7 @@
       <c r="A139" t="n">
         <v>137</v>
       </c>
-      <c r="B139" t="n">
-        <v>0</v>
-      </c>
+      <c r="B139" t="inlineStr"/>
       <c r="C139" t="n">
         <v>0</v>
       </c>
@@ -3205,6 +3399,9 @@
         <v>0</v>
       </c>
       <c r="F139" t="n">
+        <v>0</v>
+      </c>
+      <c r="G139" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3212,9 +3409,7 @@
       <c r="A140" t="n">
         <v>138</v>
       </c>
-      <c r="B140" t="n">
-        <v>0</v>
-      </c>
+      <c r="B140" t="inlineStr"/>
       <c r="C140" t="n">
         <v>0</v>
       </c>
@@ -3225,6 +3420,9 @@
         <v>0</v>
       </c>
       <c r="F140" t="n">
+        <v>0</v>
+      </c>
+      <c r="G140" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3233,7 +3431,7 @@
         <v>139</v>
       </c>
       <c r="B141" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="C141" t="n">
         <v>0</v>
@@ -3245,6 +3443,9 @@
         <v>0</v>
       </c>
       <c r="F141" t="n">
+        <v>0</v>
+      </c>
+      <c r="G141" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3252,9 +3453,7 @@
       <c r="A142" t="n">
         <v>140</v>
       </c>
-      <c r="B142" t="n">
-        <v>0</v>
-      </c>
+      <c r="B142" t="inlineStr"/>
       <c r="C142" t="n">
         <v>0</v>
       </c>
@@ -3265,6 +3464,9 @@
         <v>0</v>
       </c>
       <c r="F142" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3272,9 +3474,7 @@
       <c r="A143" t="n">
         <v>141</v>
       </c>
-      <c r="B143" t="n">
-        <v>0</v>
-      </c>
+      <c r="B143" t="inlineStr"/>
       <c r="C143" t="n">
         <v>0</v>
       </c>
@@ -3285,6 +3485,9 @@
         <v>0</v>
       </c>
       <c r="F143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3292,9 +3495,7 @@
       <c r="A144" t="n">
         <v>142</v>
       </c>
-      <c r="B144" t="n">
-        <v>0</v>
-      </c>
+      <c r="B144" t="inlineStr"/>
       <c r="C144" t="n">
         <v>0</v>
       </c>
@@ -3305,6 +3506,9 @@
         <v>0</v>
       </c>
       <c r="F144" t="n">
+        <v>0</v>
+      </c>
+      <c r="G144" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3312,9 +3516,7 @@
       <c r="A145" t="n">
         <v>143</v>
       </c>
-      <c r="B145" t="n">
-        <v>0</v>
-      </c>
+      <c r="B145" t="inlineStr"/>
       <c r="C145" t="n">
         <v>0</v>
       </c>
@@ -3325,6 +3527,9 @@
         <v>0</v>
       </c>
       <c r="F145" t="n">
+        <v>0</v>
+      </c>
+      <c r="G145" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3333,7 +3538,7 @@
         <v>144</v>
       </c>
       <c r="B146" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="C146" t="n">
         <v>0</v>
@@ -3345,6 +3550,9 @@
         <v>0</v>
       </c>
       <c r="F146" t="n">
+        <v>0</v>
+      </c>
+      <c r="G146" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3352,9 +3560,7 @@
       <c r="A147" t="n">
         <v>145</v>
       </c>
-      <c r="B147" t="n">
-        <v>0</v>
-      </c>
+      <c r="B147" t="inlineStr"/>
       <c r="C147" t="n">
         <v>0</v>
       </c>
@@ -3365,6 +3571,9 @@
         <v>0</v>
       </c>
       <c r="F147" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3372,19 +3581,20 @@
       <c r="A148" t="n">
         <v>146</v>
       </c>
-      <c r="B148" t="n">
-        <v>0</v>
-      </c>
+      <c r="B148" t="inlineStr"/>
       <c r="C148" t="n">
+        <v>0</v>
+      </c>
+      <c r="D148" t="n">
         <v>0.198</v>
       </c>
-      <c r="D148" t="n">
-        <v>0</v>
-      </c>
       <c r="E148" t="n">
         <v>0</v>
       </c>
       <c r="F148" t="n">
+        <v>0</v>
+      </c>
+      <c r="G148" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3392,9 +3602,7 @@
       <c r="A149" t="n">
         <v>147</v>
       </c>
-      <c r="B149" t="n">
-        <v>0</v>
-      </c>
+      <c r="B149" t="inlineStr"/>
       <c r="C149" t="n">
         <v>0</v>
       </c>
@@ -3405,6 +3613,9 @@
         <v>0</v>
       </c>
       <c r="F149" t="n">
+        <v>0</v>
+      </c>
+      <c r="G149" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3412,9 +3623,7 @@
       <c r="A150" t="n">
         <v>148</v>
       </c>
-      <c r="B150" t="n">
-        <v>0</v>
-      </c>
+      <c r="B150" t="inlineStr"/>
       <c r="C150" t="n">
         <v>0</v>
       </c>
@@ -3425,6 +3634,9 @@
         <v>0</v>
       </c>
       <c r="F150" t="n">
+        <v>0</v>
+      </c>
+      <c r="G150" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3433,7 +3645,7 @@
         <v>149</v>
       </c>
       <c r="B151" t="n">
-        <v>0</v>
+        <v>6.2</v>
       </c>
       <c r="C151" t="n">
         <v>0</v>
@@ -3445,6 +3657,9 @@
         <v>0</v>
       </c>
       <c r="F151" t="n">
+        <v>0</v>
+      </c>
+      <c r="G151" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3452,9 +3667,7 @@
       <c r="A152" t="n">
         <v>150</v>
       </c>
-      <c r="B152" t="n">
-        <v>0</v>
-      </c>
+      <c r="B152" t="inlineStr"/>
       <c r="C152" t="n">
         <v>0</v>
       </c>
@@ -3465,6 +3678,9 @@
         <v>0</v>
       </c>
       <c r="F152" t="n">
+        <v>0</v>
+      </c>
+      <c r="G152" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3472,19 +3688,20 @@
       <c r="A153" t="n">
         <v>151</v>
       </c>
-      <c r="B153" t="n">
-        <v>0</v>
-      </c>
+      <c r="B153" t="inlineStr"/>
       <c r="C153" t="n">
+        <v>0</v>
+      </c>
+      <c r="D153" t="n">
         <v>0.27</v>
       </c>
-      <c r="D153" t="n">
-        <v>0</v>
-      </c>
       <c r="E153" t="n">
         <v>0</v>
       </c>
       <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3492,9 +3709,7 @@
       <c r="A154" t="n">
         <v>152</v>
       </c>
-      <c r="B154" t="n">
-        <v>0</v>
-      </c>
+      <c r="B154" t="inlineStr"/>
       <c r="C154" t="n">
         <v>0</v>
       </c>
@@ -3505,6 +3720,9 @@
         <v>0</v>
       </c>
       <c r="F154" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3512,9 +3730,7 @@
       <c r="A155" t="n">
         <v>153</v>
       </c>
-      <c r="B155" t="n">
-        <v>0</v>
-      </c>
+      <c r="B155" t="inlineStr"/>
       <c r="C155" t="n">
         <v>0</v>
       </c>
@@ -3525,6 +3741,9 @@
         <v>0</v>
       </c>
       <c r="F155" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3533,7 +3752,7 @@
         <v>154</v>
       </c>
       <c r="B156" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="C156" t="n">
         <v>0</v>
@@ -3545,6 +3764,9 @@
         <v>0</v>
       </c>
       <c r="F156" t="n">
+        <v>0</v>
+      </c>
+      <c r="G156" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3552,9 +3774,7 @@
       <c r="A157" t="n">
         <v>155</v>
       </c>
-      <c r="B157" t="n">
-        <v>0</v>
-      </c>
+      <c r="B157" t="inlineStr"/>
       <c r="C157" t="n">
         <v>0</v>
       </c>
@@ -3565,6 +3785,9 @@
         <v>0</v>
       </c>
       <c r="F157" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3572,19 +3795,20 @@
       <c r="A158" t="n">
         <v>156</v>
       </c>
-      <c r="B158" t="n">
-        <v>0</v>
-      </c>
+      <c r="B158" t="inlineStr"/>
       <c r="C158" t="n">
+        <v>0</v>
+      </c>
+      <c r="D158" t="n">
         <v>0.85</v>
       </c>
-      <c r="D158" t="n">
-        <v>0</v>
-      </c>
       <c r="E158" t="n">
         <v>0</v>
       </c>
       <c r="F158" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3592,9 +3816,7 @@
       <c r="A159" t="n">
         <v>157</v>
       </c>
-      <c r="B159" t="n">
-        <v>0</v>
-      </c>
+      <c r="B159" t="inlineStr"/>
       <c r="C159" t="n">
         <v>0</v>
       </c>
@@ -3605,6 +3827,9 @@
         <v>0</v>
       </c>
       <c r="F159" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3612,9 +3837,7 @@
       <c r="A160" t="n">
         <v>158</v>
       </c>
-      <c r="B160" t="n">
-        <v>0</v>
-      </c>
+      <c r="B160" t="inlineStr"/>
       <c r="C160" t="n">
         <v>0</v>
       </c>
@@ -3625,6 +3848,9 @@
         <v>0</v>
       </c>
       <c r="F160" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3633,7 +3859,7 @@
         <v>159</v>
       </c>
       <c r="B161" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="C161" t="n">
         <v>0</v>
@@ -3645,6 +3871,9 @@
         <v>0</v>
       </c>
       <c r="F161" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3652,9 +3881,7 @@
       <c r="A162" t="n">
         <v>160</v>
       </c>
-      <c r="B162" t="n">
-        <v>0</v>
-      </c>
+      <c r="B162" t="inlineStr"/>
       <c r="C162" t="n">
         <v>0</v>
       </c>
@@ -3665,6 +3892,9 @@
         <v>0</v>
       </c>
       <c r="F162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G162" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3672,9 +3902,7 @@
       <c r="A163" t="n">
         <v>161</v>
       </c>
-      <c r="B163" t="n">
-        <v>0</v>
-      </c>
+      <c r="B163" t="inlineStr"/>
       <c r="C163" t="n">
         <v>0</v>
       </c>
@@ -3685,6 +3913,9 @@
         <v>0</v>
       </c>
       <c r="F163" t="n">
+        <v>0</v>
+      </c>
+      <c r="G163" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3692,9 +3923,7 @@
       <c r="A164" t="n">
         <v>162</v>
       </c>
-      <c r="B164" t="n">
-        <v>0</v>
-      </c>
+      <c r="B164" t="inlineStr"/>
       <c r="C164" t="n">
         <v>0</v>
       </c>
@@ -3705,6 +3934,9 @@
         <v>0</v>
       </c>
       <c r="F164" t="n">
+        <v>0</v>
+      </c>
+      <c r="G164" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3712,9 +3944,7 @@
       <c r="A165" t="n">
         <v>163</v>
       </c>
-      <c r="B165" t="n">
-        <v>0</v>
-      </c>
+      <c r="B165" t="inlineStr"/>
       <c r="C165" t="n">
         <v>0</v>
       </c>
@@ -3725,6 +3955,9 @@
         <v>0</v>
       </c>
       <c r="F165" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3733,7 +3966,7 @@
         <v>164</v>
       </c>
       <c r="B166" t="n">
-        <v>0</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C166" t="n">
         <v>0</v>
@@ -3745,6 +3978,9 @@
         <v>0</v>
       </c>
       <c r="F166" t="n">
+        <v>0</v>
+      </c>
+      <c r="G166" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3752,9 +3988,7 @@
       <c r="A167" t="n">
         <v>165</v>
       </c>
-      <c r="B167" t="n">
-        <v>0</v>
-      </c>
+      <c r="B167" t="inlineStr"/>
       <c r="C167" t="n">
         <v>0</v>
       </c>
@@ -3765,6 +3999,9 @@
         <v>0</v>
       </c>
       <c r="F167" t="n">
+        <v>0</v>
+      </c>
+      <c r="G167" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3772,9 +4009,7 @@
       <c r="A168" t="n">
         <v>166</v>
       </c>
-      <c r="B168" t="n">
-        <v>0</v>
-      </c>
+      <c r="B168" t="inlineStr"/>
       <c r="C168" t="n">
         <v>0</v>
       </c>
@@ -3785,6 +4020,9 @@
         <v>0</v>
       </c>
       <c r="F168" t="n">
+        <v>0</v>
+      </c>
+      <c r="G168" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3792,9 +4030,7 @@
       <c r="A169" t="n">
         <v>167</v>
       </c>
-      <c r="B169" t="n">
-        <v>0</v>
-      </c>
+      <c r="B169" t="inlineStr"/>
       <c r="C169" t="n">
         <v>0</v>
       </c>
@@ -3805,6 +4041,9 @@
         <v>0</v>
       </c>
       <c r="F169" t="n">
+        <v>0</v>
+      </c>
+      <c r="G169" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3812,9 +4051,7 @@
       <c r="A170" t="n">
         <v>168</v>
       </c>
-      <c r="B170" t="n">
-        <v>0</v>
-      </c>
+      <c r="B170" t="inlineStr"/>
       <c r="C170" t="n">
         <v>0</v>
       </c>
@@ -3825,6 +4062,9 @@
         <v>0</v>
       </c>
       <c r="F170" t="n">
+        <v>0</v>
+      </c>
+      <c r="G170" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3833,7 +4073,7 @@
         <v>169</v>
       </c>
       <c r="B171" t="n">
-        <v>0</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="C171" t="n">
         <v>0</v>
@@ -3845,6 +4085,9 @@
         <v>0</v>
       </c>
       <c r="F171" t="n">
+        <v>0</v>
+      </c>
+      <c r="G171" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3852,9 +4095,7 @@
       <c r="A172" t="n">
         <v>170</v>
       </c>
-      <c r="B172" t="n">
-        <v>0</v>
-      </c>
+      <c r="B172" t="inlineStr"/>
       <c r="C172" t="n">
         <v>0</v>
       </c>
@@ -3865,6 +4106,9 @@
         <v>0</v>
       </c>
       <c r="F172" t="n">
+        <v>0</v>
+      </c>
+      <c r="G172" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3872,9 +4116,7 @@
       <c r="A173" t="n">
         <v>171</v>
       </c>
-      <c r="B173" t="n">
-        <v>0</v>
-      </c>
+      <c r="B173" t="inlineStr"/>
       <c r="C173" t="n">
         <v>0</v>
       </c>
@@ -3885,6 +4127,9 @@
         <v>0</v>
       </c>
       <c r="F173" t="n">
+        <v>0</v>
+      </c>
+      <c r="G173" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3892,9 +4137,7 @@
       <c r="A174" t="n">
         <v>172</v>
       </c>
-      <c r="B174" t="n">
-        <v>0</v>
-      </c>
+      <c r="B174" t="inlineStr"/>
       <c r="C174" t="n">
         <v>0</v>
       </c>
@@ -3905,6 +4148,9 @@
         <v>0</v>
       </c>
       <c r="F174" t="n">
+        <v>0</v>
+      </c>
+      <c r="G174" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3912,9 +4158,7 @@
       <c r="A175" t="n">
         <v>173</v>
       </c>
-      <c r="B175" t="n">
-        <v>0</v>
-      </c>
+      <c r="B175" t="inlineStr"/>
       <c r="C175" t="n">
         <v>0</v>
       </c>
@@ -3925,6 +4169,9 @@
         <v>0</v>
       </c>
       <c r="F175" t="n">
+        <v>0</v>
+      </c>
+      <c r="G175" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3933,7 +4180,7 @@
         <v>174</v>
       </c>
       <c r="B176" t="n">
-        <v>0</v>
+        <v>9.4</v>
       </c>
       <c r="C176" t="n">
         <v>0</v>
@@ -3945,6 +4192,9 @@
         <v>0</v>
       </c>
       <c r="F176" t="n">
+        <v>0</v>
+      </c>
+      <c r="G176" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3952,9 +4202,7 @@
       <c r="A177" t="n">
         <v>175</v>
       </c>
-      <c r="B177" t="n">
-        <v>0</v>
-      </c>
+      <c r="B177" t="inlineStr"/>
       <c r="C177" t="n">
         <v>0</v>
       </c>
@@ -3965,6 +4213,9 @@
         <v>0</v>
       </c>
       <c r="F177" t="n">
+        <v>0</v>
+      </c>
+      <c r="G177" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3972,9 +4223,7 @@
       <c r="A178" t="n">
         <v>176</v>
       </c>
-      <c r="B178" t="n">
-        <v>0</v>
-      </c>
+      <c r="B178" t="inlineStr"/>
       <c r="C178" t="n">
         <v>0</v>
       </c>
@@ -3985,6 +4234,9 @@
         <v>0</v>
       </c>
       <c r="F178" t="n">
+        <v>0</v>
+      </c>
+      <c r="G178" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3992,9 +4244,7 @@
       <c r="A179" t="n">
         <v>177</v>
       </c>
-      <c r="B179" t="n">
-        <v>0</v>
-      </c>
+      <c r="B179" t="inlineStr"/>
       <c r="C179" t="n">
         <v>0</v>
       </c>
@@ -4005,6 +4255,9 @@
         <v>0</v>
       </c>
       <c r="F179" t="n">
+        <v>0</v>
+      </c>
+      <c r="G179" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4012,9 +4265,7 @@
       <c r="A180" t="n">
         <v>178</v>
       </c>
-      <c r="B180" t="n">
-        <v>0</v>
-      </c>
+      <c r="B180" t="inlineStr"/>
       <c r="C180" t="n">
         <v>0</v>
       </c>
@@ -4025,6 +4276,9 @@
         <v>0</v>
       </c>
       <c r="F180" t="n">
+        <v>0</v>
+      </c>
+      <c r="G180" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4033,7 +4287,7 @@
         <v>179</v>
       </c>
       <c r="B181" t="n">
-        <v>0</v>
+        <v>10.1</v>
       </c>
       <c r="C181" t="n">
         <v>0</v>
@@ -4045,6 +4299,9 @@
         <v>0</v>
       </c>
       <c r="F181" t="n">
+        <v>0</v>
+      </c>
+      <c r="G181" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4052,9 +4309,7 @@
       <c r="A182" t="n">
         <v>180</v>
       </c>
-      <c r="B182" t="n">
-        <v>0</v>
-      </c>
+      <c r="B182" t="inlineStr"/>
       <c r="C182" t="n">
         <v>0</v>
       </c>
@@ -4065,6 +4320,9 @@
         <v>0</v>
       </c>
       <c r="F182" t="n">
+        <v>0</v>
+      </c>
+      <c r="G182" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>